<commit_message>
Added RDA for cut-off of least polluted sites.
</commit_message>
<xml_diff>
--- a/results/01_pollution_assessment/tables/MaxRel_site_rankings.xlsx
+++ b/results/01_pollution_assessment/tables/MaxRel_site_rankings.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4279270434436434</v>
+        <v>0.4279270434436436</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.4452953699698398</v>
+        <v>0.44529536996984</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.4499061108660709</v>
+        <v>0.4499061108660707</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.4566228460312882</v>
+        <v>0.4566228460312883</v>
       </c>
       <c r="D6" t="n">
         <v>5</v>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.4643361686496821</v>
+        <v>0.4643361686496823</v>
       </c>
       <c r="D7" t="n">
         <v>6</v>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.4645219119572452</v>
+        <v>0.4645219119572454</v>
       </c>
       <c r="D8" t="n">
         <v>7</v>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.4668088778224345</v>
+        <v>0.4668088778224347</v>
       </c>
       <c r="D9" t="n">
         <v>8</v>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.4767018754778721</v>
+        <v>0.4767018754778722</v>
       </c>
       <c r="D12" t="n">
         <v>11</v>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.4785962151959065</v>
+        <v>0.4785962151959063</v>
       </c>
       <c r="D13" t="n">
         <v>12</v>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.4816008485980839</v>
+        <v>0.4816008485980842</v>
       </c>
       <c r="D14" t="n">
         <v>13</v>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.4817703950445548</v>
+        <v>0.4817703950445553</v>
       </c>
       <c r="D15" t="n">
         <v>14</v>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.484952423083475</v>
+        <v>0.4849524230834752</v>
       </c>
       <c r="D17" t="n">
         <v>16</v>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.4852841580118419</v>
+        <v>0.4852841580118421</v>
       </c>
       <c r="D18" t="n">
         <v>17</v>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.4854230154784182</v>
+        <v>0.4854230154784185</v>
       </c>
       <c r="D19" t="n">
         <v>18</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.4917373475281424</v>
+        <v>0.4917373475281425</v>
       </c>
       <c r="D20" t="n">
         <v>19</v>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.4920495726049761</v>
+        <v>0.4920495726049763</v>
       </c>
       <c r="D21" t="n">
         <v>20</v>
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.4977908434553533</v>
+        <v>0.4977908434553531</v>
       </c>
       <c r="D22" t="n">
         <v>21</v>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.4986068132440482</v>
+        <v>0.4986068132440484</v>
       </c>
       <c r="D23" t="n">
         <v>22</v>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.4996454746195236</v>
+        <v>0.4996454746195239</v>
       </c>
       <c r="D24" t="n">
         <v>23</v>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.5005856599216519</v>
+        <v>0.500585659921652</v>
       </c>
       <c r="D27" t="n">
         <v>26</v>
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.5024228727994454</v>
+        <v>0.5024228727994456</v>
       </c>
       <c r="D29" t="n">
         <v>28</v>
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.5032146687493856</v>
+        <v>0.5032146687493858</v>
       </c>
       <c r="D30" t="n">
         <v>29</v>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.5104225059758862</v>
+        <v>0.5104225059758865</v>
       </c>
       <c r="D31" t="n">
         <v>30</v>
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.5115589970868325</v>
+        <v>0.5115589970868324</v>
       </c>
       <c r="D32" t="n">
         <v>31</v>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.5127327830639198</v>
+        <v>0.51273278306392</v>
       </c>
       <c r="D33" t="n">
         <v>32</v>
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.5163819878358257</v>
+        <v>0.5163819878358256</v>
       </c>
       <c r="D35" t="n">
         <v>34</v>
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.5184533233839834</v>
+        <v>0.5184533233839833</v>
       </c>
       <c r="D36" t="n">
         <v>35</v>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.5186062015990544</v>
+        <v>0.5186062015990545</v>
       </c>
       <c r="D37" t="n">
         <v>36</v>
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.5203593278017669</v>
+        <v>0.5203593278017671</v>
       </c>
       <c r="D38" t="n">
         <v>37</v>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.5209571937133598</v>
+        <v>0.52095719371336</v>
       </c>
       <c r="D39" t="n">
         <v>38</v>
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.5227822636279221</v>
+        <v>0.5227822636279224</v>
       </c>
       <c r="D41" t="n">
         <v>40</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.5228091805623424</v>
+        <v>0.5228091805623426</v>
       </c>
       <c r="D42" t="n">
         <v>41</v>
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.5254974249028412</v>
+        <v>0.5254974249028411</v>
       </c>
       <c r="D44" t="n">
         <v>43</v>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.5399745325352203</v>
+        <v>0.5399745325352201</v>
       </c>
       <c r="D45" t="n">
         <v>44</v>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.5422080833277145</v>
+        <v>0.5422080833277143</v>
       </c>
       <c r="D46" t="n">
         <v>45</v>
@@ -1175,7 +1175,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.5424472754850664</v>
+        <v>0.5424472754850667</v>
       </c>
       <c r="D47" t="n">
         <v>46</v>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.5475103983506402</v>
+        <v>0.54751039835064</v>
       </c>
       <c r="D48" t="n">
         <v>47</v>
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.5503133858873539</v>
+        <v>0.5503133858873541</v>
       </c>
       <c r="D49" t="n">
         <v>48</v>
@@ -1223,7 +1223,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.5513697836534377</v>
+        <v>0.551369783653438</v>
       </c>
       <c r="D50" t="n">
         <v>49</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.5561563520250102</v>
+        <v>0.5561563520250101</v>
       </c>
       <c r="D51" t="n">
         <v>50</v>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.5576156513591051</v>
+        <v>0.5576156513591055</v>
       </c>
       <c r="D52" t="n">
         <v>51</v>
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.5579190477234698</v>
+        <v>0.5579190477234697</v>
       </c>
       <c r="D53" t="n">
         <v>52</v>
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.5601275943142237</v>
+        <v>0.5601275943142239</v>
       </c>
       <c r="D54" t="n">
         <v>53</v>
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0.5640676320858971</v>
+        <v>0.5640676320858974</v>
       </c>
       <c r="D56" t="n">
         <v>55</v>
@@ -1399,7 +1399,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0.5722068049985606</v>
+        <v>0.5722068049985605</v>
       </c>
       <c r="D61" t="n">
         <v>60</v>
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0.5724960596840994</v>
+        <v>0.5724960596840993</v>
       </c>
       <c r="D62" t="n">
         <v>61</v>
@@ -1431,7 +1431,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0.5744726564412542</v>
+        <v>0.5744726564412541</v>
       </c>
       <c r="D63" t="n">
         <v>62</v>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0.5775632142418805</v>
+        <v>0.5775632142418804</v>
       </c>
       <c r="D65" t="n">
         <v>64</v>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0.5804986749188547</v>
+        <v>0.5804986749188545</v>
       </c>
       <c r="D67" t="n">
         <v>66</v>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.5856717489409903</v>
+        <v>0.5856717489409905</v>
       </c>
       <c r="D69" t="n">
         <v>68</v>
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.5899256148787306</v>
+        <v>0.5899256148787307</v>
       </c>
       <c r="D71" t="n">
         <v>70</v>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.5926706541324308</v>
+        <v>0.5926706541324307</v>
       </c>
       <c r="D72" t="n">
         <v>71</v>
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.5930481878495744</v>
+        <v>0.5930481878495745</v>
       </c>
       <c r="D73" t="n">
         <v>72</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.603074929859872</v>
+        <v>0.6030749298598718</v>
       </c>
       <c r="D79" t="n">
         <v>78</v>
@@ -1719,7 +1719,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.6076986464554137</v>
+        <v>0.6076986464554136</v>
       </c>
       <c r="D81" t="n">
         <v>80</v>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.6084478435480961</v>
+        <v>0.608447843548096</v>
       </c>
       <c r="D82" t="n">
         <v>81</v>
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>0.6110652922305252</v>
+        <v>0.6110652922305251</v>
       </c>
       <c r="D83" t="n">
         <v>82</v>
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.6129973684613884</v>
+        <v>0.6129973684613883</v>
       </c>
       <c r="D85" t="n">
         <v>84</v>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.6146018592525765</v>
+        <v>0.6146018592525763</v>
       </c>
       <c r="D86" t="n">
         <v>85</v>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>0.6154034604025812</v>
+        <v>0.615403460402581</v>
       </c>
       <c r="D87" t="n">
         <v>86</v>
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>0.6168109707877535</v>
+        <v>0.6168109707877533</v>
       </c>
       <c r="D88" t="n">
         <v>87</v>
@@ -1863,7 +1863,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>0.6178038292714395</v>
+        <v>0.6178038292714398</v>
       </c>
       <c r="D90" t="n">
         <v>89</v>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>0.6185465476509819</v>
+        <v>0.6185465476509818</v>
       </c>
       <c r="D91" t="n">
         <v>90</v>
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0.6213889412428641</v>
+        <v>0.621388941242864</v>
       </c>
       <c r="D93" t="n">
         <v>92</v>
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>0.625912350805265</v>
+        <v>0.6259123508052651</v>
       </c>
       <c r="D95" t="n">
         <v>94</v>
@@ -1959,7 +1959,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>0.6261505446070396</v>
+        <v>0.6261505446070393</v>
       </c>
       <c r="D96" t="n">
         <v>95</v>
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>0.6276808832828212</v>
+        <v>0.6276808832828213</v>
       </c>
       <c r="D97" t="n">
         <v>96</v>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>0.6280847762652918</v>
+        <v>0.6280847762652917</v>
       </c>
       <c r="D98" t="n">
         <v>97</v>
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.6300470945975647</v>
+        <v>0.6300470945975645</v>
       </c>
       <c r="D99" t="n">
         <v>98</v>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>0.6335293202176466</v>
+        <v>0.6335293202176467</v>
       </c>
       <c r="D100" t="n">
         <v>99</v>
@@ -2039,7 +2039,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>0.6337650931900197</v>
+        <v>0.6337650931900195</v>
       </c>
       <c r="D101" t="n">
         <v>100</v>
@@ -2055,7 +2055,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>0.6354777360989823</v>
+        <v>0.6354777360989819</v>
       </c>
       <c r="D102" t="n">
         <v>101</v>
@@ -2071,7 +2071,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>0.6365566232118295</v>
+        <v>0.6365566232118293</v>
       </c>
       <c r="D103" t="n">
         <v>102</v>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>0.6373599866468866</v>
+        <v>0.6373599866468865</v>
       </c>
       <c r="D104" t="n">
         <v>103</v>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>0.6374505489593454</v>
+        <v>0.6374505489593453</v>
       </c>
       <c r="D105" t="n">
         <v>104</v>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>0.6409648891583338</v>
+        <v>0.6409648891583339</v>
       </c>
       <c r="D106" t="n">
         <v>105</v>
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>0.6462142951592343</v>
+        <v>0.6462142951592346</v>
       </c>
       <c r="D109" t="n">
         <v>108</v>
@@ -2183,7 +2183,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>0.646864932675818</v>
+        <v>0.6468649326758181</v>
       </c>
       <c r="D110" t="n">
         <v>109</v>
@@ -2215,7 +2215,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>0.6478839196008841</v>
+        <v>0.647883919600884</v>
       </c>
       <c r="D112" t="n">
         <v>111</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>0.6512301012218443</v>
+        <v>0.6512301012218442</v>
       </c>
       <c r="D115" t="n">
         <v>114</v>
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>0.6590007243578806</v>
+        <v>0.6590007243578807</v>
       </c>
       <c r="D116" t="n">
         <v>115</v>
@@ -2295,7 +2295,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>0.6705968300910684</v>
+        <v>0.6705968300910682</v>
       </c>
       <c r="D117" t="n">
         <v>116</v>
@@ -2311,7 +2311,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>0.6795732758109243</v>
+        <v>0.6795732758109245</v>
       </c>
       <c r="D118" t="n">
         <v>117</v>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>0.6822249116624723</v>
+        <v>0.6822249116624725</v>
       </c>
       <c r="D119" t="n">
         <v>118</v>
@@ -2343,7 +2343,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>0.6853216505185022</v>
+        <v>0.6853216505185021</v>
       </c>
       <c r="D120" t="n">
         <v>119</v>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>0.6899527436386715</v>
+        <v>0.6899527436386717</v>
       </c>
       <c r="D121" t="n">
         <v>120</v>
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>0.7008729885720086</v>
+        <v>0.7008729885720087</v>
       </c>
       <c r="D125" t="n">
         <v>124</v>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>0.7052528390632292</v>
+        <v>0.7052528390632291</v>
       </c>
       <c r="D127" t="n">
         <v>126</v>
@@ -2503,7 +2503,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>0.712579390219759</v>
+        <v>0.7125793902197588</v>
       </c>
       <c r="D130" t="n">
         <v>129</v>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>0.7155209006446386</v>
+        <v>0.7155209006446385</v>
       </c>
       <c r="D131" t="n">
         <v>130</v>
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>0.7172240308022388</v>
+        <v>0.7172240308022387</v>
       </c>
       <c r="D132" t="n">
         <v>131</v>
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>0.7177302982953639</v>
+        <v>0.7177302982953641</v>
       </c>
       <c r="D133" t="n">
         <v>132</v>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>0.7300656900907722</v>
+        <v>0.730065690090772</v>
       </c>
       <c r="D135" t="n">
         <v>134</v>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>0.7317580553485201</v>
+        <v>0.73175805534852</v>
       </c>
       <c r="D137" t="n">
         <v>136</v>
@@ -2631,7 +2631,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>0.7332544448199504</v>
+        <v>0.7332544448199501</v>
       </c>
       <c r="D138" t="n">
         <v>137</v>
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>0.7357783871585788</v>
+        <v>0.7357783871585791</v>
       </c>
       <c r="D139" t="n">
         <v>138</v>
@@ -2695,7 +2695,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>0.7381203637182031</v>
+        <v>0.7381203637182029</v>
       </c>
       <c r="D142" t="n">
         <v>141</v>
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>0.7419293129378134</v>
+        <v>0.7419293129378133</v>
       </c>
       <c r="D144" t="n">
         <v>143</v>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>0.7422970234339675</v>
+        <v>0.7422970234339674</v>
       </c>
       <c r="D145" t="n">
         <v>144</v>
@@ -2791,7 +2791,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>0.7518632452480585</v>
+        <v>0.7518632452480591</v>
       </c>
       <c r="D148" t="n">
         <v>147</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>0.7549672201377287</v>
+        <v>0.7549672201377288</v>
       </c>
       <c r="D149" t="n">
         <v>148</v>
@@ -2823,7 +2823,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>0.7553621744720782</v>
+        <v>0.7553621744720783</v>
       </c>
       <c r="D150" t="n">
         <v>149</v>
@@ -2855,7 +2855,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>0.7651163916690356</v>
+        <v>0.7651163916690357</v>
       </c>
       <c r="D152" t="n">
         <v>151</v>
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>0.7667095077809323</v>
+        <v>0.7667095077809322</v>
       </c>
       <c r="D154" t="n">
         <v>153</v>
@@ -2903,7 +2903,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>0.7693003371589151</v>
+        <v>0.7693003371589152</v>
       </c>
       <c r="D155" t="n">
         <v>154</v>
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>0.7704970058097398</v>
+        <v>0.7704970058097397</v>
       </c>
       <c r="D156" t="n">
         <v>155</v>
@@ -2935,7 +2935,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>0.77131020120551</v>
+        <v>0.7713102012055102</v>
       </c>
       <c r="D157" t="n">
         <v>156</v>
@@ -2951,7 +2951,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>0.7887574063130198</v>
+        <v>0.7887574063130196</v>
       </c>
       <c r="D158" t="n">
         <v>157</v>
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>0.7891204243184647</v>
+        <v>0.7891204243184649</v>
       </c>
       <c r="D159" t="n">
         <v>158</v>
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>0.791652672702895</v>
+        <v>0.7916526727028949</v>
       </c>
       <c r="D160" t="n">
         <v>159</v>
@@ -2999,7 +2999,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>0.7918350375648093</v>
+        <v>0.7918350375648097</v>
       </c>
       <c r="D161" t="n">
         <v>160</v>
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>0.7927824614648837</v>
+        <v>0.7927824614648841</v>
       </c>
       <c r="D162" t="n">
         <v>161</v>
@@ -3031,7 +3031,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>0.7953765230546896</v>
+        <v>0.7953765230546895</v>
       </c>
       <c r="D163" t="n">
         <v>162</v>
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>0.7968850694695153</v>
+        <v>0.7968850694695152</v>
       </c>
       <c r="D164" t="n">
         <v>163</v>
@@ -3063,7 +3063,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>0.7973251537487782</v>
+        <v>0.7973251537487783</v>
       </c>
       <c r="D165" t="n">
         <v>164</v>
@@ -3079,7 +3079,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>0.7992003819160949</v>
+        <v>0.7992003819160945</v>
       </c>
       <c r="D166" t="n">
         <v>165</v>
@@ -3095,7 +3095,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>0.8010756606369889</v>
+        <v>0.8010756606369891</v>
       </c>
       <c r="D167" t="n">
         <v>166</v>
@@ -3111,7 +3111,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>0.8016283830315825</v>
+        <v>0.8016283830315827</v>
       </c>
       <c r="D168" t="n">
         <v>167</v>
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>0.8068000919688815</v>
+        <v>0.8068000919688813</v>
       </c>
       <c r="D169" t="n">
         <v>168</v>
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>0.8082516259482172</v>
+        <v>0.8082516259482169</v>
       </c>
       <c r="D170" t="n">
         <v>169</v>
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>0.8095796148110737</v>
+        <v>0.8095796148110739</v>
       </c>
       <c r="D171" t="n">
         <v>170</v>
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>0.8117628853166764</v>
+        <v>0.8117628853166763</v>
       </c>
       <c r="D172" t="n">
         <v>171</v>
@@ -3223,7 +3223,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>0.8170967647078101</v>
+        <v>0.8170967647078108</v>
       </c>
       <c r="D175" t="n">
         <v>174</v>
@@ -3239,7 +3239,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>0.819192150054835</v>
+        <v>0.8191921500548353</v>
       </c>
       <c r="D176" t="n">
         <v>175</v>
@@ -3271,7 +3271,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>0.8229620343245406</v>
+        <v>0.8229620343245404</v>
       </c>
       <c r="D178" t="n">
         <v>177</v>
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>0.8253991727079085</v>
+        <v>0.825399172707909</v>
       </c>
       <c r="D179" t="n">
         <v>178</v>
@@ -3303,7 +3303,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>0.8256982409959298</v>
+        <v>0.8256982409959301</v>
       </c>
       <c r="D180" t="n">
         <v>179</v>
@@ -3319,7 +3319,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>0.830568356786174</v>
+        <v>0.8305683567861738</v>
       </c>
       <c r="D181" t="n">
         <v>180</v>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>0.8330840616624919</v>
+        <v>0.8330840616624922</v>
       </c>
       <c r="D182" t="n">
         <v>181</v>
@@ -3351,7 +3351,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>0.834081369310496</v>
+        <v>0.8340813693104963</v>
       </c>
       <c r="D183" t="n">
         <v>182</v>
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>0.836022752643399</v>
+        <v>0.8360227526433988</v>
       </c>
       <c r="D184" t="n">
         <v>183</v>
@@ -3383,7 +3383,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>0.8371829803608046</v>
+        <v>0.8371829803608051</v>
       </c>
       <c r="D185" t="n">
         <v>184</v>
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>0.8377669859084637</v>
+        <v>0.837766985908464</v>
       </c>
       <c r="D186" t="n">
         <v>185</v>
@@ -3415,7 +3415,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>0.8402115464951354</v>
+        <v>0.8402115464951359</v>
       </c>
       <c r="D187" t="n">
         <v>186</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>0.8404195797588516</v>
+        <v>0.8404195797588517</v>
       </c>
       <c r="D188" t="n">
         <v>187</v>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>0.8462082812769164</v>
+        <v>0.8462082812769163</v>
       </c>
       <c r="D189" t="n">
         <v>188</v>
@@ -3463,7 +3463,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>0.8479939113629964</v>
+        <v>0.8479939113629967</v>
       </c>
       <c r="D190" t="n">
         <v>189</v>
@@ -3479,7 +3479,7 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>0.8493559187984098</v>
+        <v>0.8493559187984099</v>
       </c>
       <c r="D191" t="n">
         <v>190</v>
@@ -3495,7 +3495,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>0.8498365014758507</v>
+        <v>0.8498365014758508</v>
       </c>
       <c r="D192" t="n">
         <v>191</v>
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>0.8684307388725729</v>
+        <v>0.868430738872573</v>
       </c>
       <c r="D193" t="n">
         <v>192</v>
@@ -3527,7 +3527,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>0.8693874790905177</v>
+        <v>0.8693874790905182</v>
       </c>
       <c r="D194" t="n">
         <v>193</v>
@@ -3543,7 +3543,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>0.8696275423735416</v>
+        <v>0.869627542373542</v>
       </c>
       <c r="D195" t="n">
         <v>194</v>
@@ -3559,7 +3559,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>0.8697147900844762</v>
+        <v>0.8697147900844761</v>
       </c>
       <c r="D196" t="n">
         <v>195</v>
@@ -3575,7 +3575,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>0.8719927416615398</v>
+        <v>0.8719927416615396</v>
       </c>
       <c r="D197" t="n">
         <v>196</v>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>0.8723671399685544</v>
+        <v>0.8723671399685542</v>
       </c>
       <c r="D198" t="n">
         <v>197</v>
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>0.8776809367945191</v>
+        <v>0.877680936794519</v>
       </c>
       <c r="D199" t="n">
         <v>198</v>
@@ -3639,7 +3639,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>0.8822790391143867</v>
+        <v>0.8822790391143869</v>
       </c>
       <c r="D201" t="n">
         <v>200</v>
@@ -3655,7 +3655,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>0.889267526655467</v>
+        <v>0.8892675266554667</v>
       </c>
       <c r="D202" t="n">
         <v>201</v>
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>0.9034678722125055</v>
+        <v>0.9034678722125057</v>
       </c>
       <c r="D204" t="n">
         <v>203</v>
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>0.9115225033341499</v>
+        <v>0.9115225033341503</v>
       </c>
       <c r="D205" t="n">
         <v>204</v>
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>0.9165246489772899</v>
+        <v>0.9165246489772896</v>
       </c>
       <c r="D206" t="n">
         <v>205</v>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>0.9215996131933117</v>
+        <v>0.9215996131933122</v>
       </c>
       <c r="D207" t="n">
         <v>206</v>
@@ -3751,7 +3751,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>0.923814068391583</v>
+        <v>0.9238140683915834</v>
       </c>
       <c r="D208" t="n">
         <v>207</v>
@@ -3767,7 +3767,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>0.9243267853069075</v>
+        <v>0.9243267853069079</v>
       </c>
       <c r="D209" t="n">
         <v>208</v>
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>0.9272890782070158</v>
+        <v>0.9272890782070157</v>
       </c>
       <c r="D210" t="n">
         <v>209</v>
@@ -3799,7 +3799,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>0.9334990011324412</v>
+        <v>0.9334990011324414</v>
       </c>
       <c r="D211" t="n">
         <v>210</v>
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>0.9395089289547327</v>
+        <v>0.9395089289547325</v>
       </c>
       <c r="D212" t="n">
         <v>211</v>
@@ -3831,7 +3831,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>0.9423048753384816</v>
+        <v>0.9423048753384821</v>
       </c>
       <c r="D213" t="n">
         <v>212</v>
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>0.9444986096343727</v>
+        <v>0.944498609634373</v>
       </c>
       <c r="D214" t="n">
         <v>213</v>
@@ -3863,7 +3863,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>0.9502781173816847</v>
+        <v>0.9502781173816849</v>
       </c>
       <c r="D215" t="n">
         <v>214</v>
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>0.9508253203478138</v>
+        <v>0.9508253203478136</v>
       </c>
       <c r="D216" t="n">
         <v>215</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>0.9521524407998946</v>
+        <v>0.9521524407998949</v>
       </c>
       <c r="D217" t="n">
         <v>216</v>
@@ -3911,7 +3911,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>0.9521888956593905</v>
+        <v>0.9521888956593909</v>
       </c>
       <c r="D218" t="n">
         <v>217</v>
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>0.9533573171392666</v>
+        <v>0.9533573171392671</v>
       </c>
       <c r="D219" t="n">
         <v>218</v>
@@ -3943,7 +3943,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>0.9557272924072273</v>
+        <v>0.9557272924072274</v>
       </c>
       <c r="D220" t="n">
         <v>219</v>
@@ -3959,7 +3959,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>0.9558323625751309</v>
+        <v>0.9558323625751313</v>
       </c>
       <c r="D221" t="n">
         <v>220</v>
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>0.9585577371642899</v>
+        <v>0.9585577371642903</v>
       </c>
       <c r="D222" t="n">
         <v>221</v>
@@ -3991,7 +3991,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>0.9597483543529494</v>
+        <v>0.9597483543529495</v>
       </c>
       <c r="D223" t="n">
         <v>222</v>
@@ -4055,7 +4055,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>0.9775067813330917</v>
+        <v>0.9775067813330918</v>
       </c>
       <c r="D227" t="n">
         <v>226</v>
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>0.9779984231567342</v>
+        <v>0.9779984231567345</v>
       </c>
       <c r="D228" t="n">
         <v>227</v>
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>0.9905182490356108</v>
+        <v>0.9905182490356109</v>
       </c>
       <c r="D229" t="n">
         <v>228</v>

</xml_diff>